<commit_message>
FIX: Adds a regression test
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/LOOKUP_AND_REFERENCE/XMATCH.xlsx
+++ b/xlsx/tests/calc_tests/LOOKUP_AND_REFERENCE/XMATCH.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nhatcher/Documents/Excel/LOOKUP_AND_REFERENCE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BACE2F8D-C0A4-E64F-B4E1-6636EE4CEA2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EAAAEC9-0CAC-8245-A099-9768B81FF9B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2780" yWindow="1580" windowWidth="28040" windowHeight="17180" xr2:uid="{C998B8C6-C02F-8643-B940-8BB9636E6049}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
   <si>
     <t>Country</t>
   </si>
@@ -91,6 +91,12 @@
   </si>
   <si>
     <t>Francialy</t>
+  </si>
+  <si>
+    <t>apple</t>
+  </si>
+  <si>
+    <t>bannana</t>
   </si>
 </sst>
 </file>
@@ -462,7 +468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6BA73AF-2076-564D-AE0C-E0B316977689}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -547,6 +553,20 @@
         <v>9</v>
       </c>
     </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" t="e">
+        <f>_xlfn.XMATCH(42,A14:A15,3)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>